<commit_message>
KPI cards: titles as constant fields so the label text is editable
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142KX8kgH6uvyxTRm3Mumhx
</commit_message>
<xml_diff>
--- a/docs/Arcadia_KPI_Cards_Config.xlsx
+++ b/docs/Arcadia_KPI_Cards_Config.xlsx
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1087,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1927,6 +1926,91 @@
       <c r="C51" s="3" t="inlineStr">
         <is>
           <t>calibration only</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>KPI 1 Title</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>"Closing headcount"</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>constant text for the title layer's Label shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>KPI 2 Title</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>"Closing FTE"</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>constant text for the title layer's Label shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>KPI 3 Title</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>"Hires"</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>constant text for the title layer's Label shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>KPI 4 Title</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>"Voluntary turnover (annualized)"</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>constant text for the title layer's Label shelf</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>KPI 5 Title</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>"Internal moves"</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>constant text for the title layer's Label shelf</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2110,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Label text (typed): Closing headcount</t>
+          <t>Label field: KPI 1 Title</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -2186,7 +2270,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Label text (typed): Closing FTE</t>
+          <t>Label field: KPI 2 Title</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2282,7 +2366,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Label text (typed): Hires</t>
+          <t>Label field: KPI 3 Title</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -2378,7 +2462,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Label text (typed): Voluntary turnover (annualized)</t>
+          <t>Label field: KPI 4 Title</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -2474,7 +2558,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Label text (typed): Internal moves</t>
+          <t>Label field: KPI 5 Title</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">

</xml_diff>

<commit_message>
KPI cards: size is set on the dashboard, card 1 note in one layer
</commit_message>
<xml_diff>
--- a/docs/Arcadia_KPI_Cards_Config.xlsx
+++ b/docs/Arcadia_KPI_Cards_Config.xlsx
@@ -2025,7 +2025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2159,7 +2159,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Note 1 Up</t>
+          <t>Note 1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 1 Note Up</t>
+          <t>Label fields on one line: KPI 1 Note Up, KPI 1 Note Down, KPI 1 Note Flat</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -2184,19 +2184,19 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>#006B66</t>
+          <t>Up #006B66 / Down #B8401F / Flat #5A6170 (color each field)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Note 1 Down</t>
+          <t>Title 2</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 1</t>
+          <t>kpi_pt Title 2</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -2206,29 +2206,29 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 1 Note Down</t>
+          <t>Label field: KPI 2 Title</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Tableau Book 8pt</t>
+          <t>Tableau Semibold 8pt</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>#B8401F</t>
+          <t>#5A6170</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Note 1 Flat</t>
+          <t>Value 2</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 1</t>
+          <t>kpi_pt Value 2</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -2238,29 +2238,29 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 1 Note Flat</t>
+          <t>Label field: KPI 2 Value</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Tableau Book 8pt</t>
+          <t>Tableau Bold 20pt</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>#5A6170</t>
+          <t>#13233A</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Title 2</t>
+          <t>Note 2</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 2</t>
+          <t>kpi_pt Note 2</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -2270,12 +2270,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 2 Title</t>
+          <t>Label field: KPI 2 Note</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Tableau Semibold 8pt</t>
+          <t>Tableau Book 8pt</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -2287,12 +2287,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Value 2</t>
+          <t>Title 3</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 2</t>
+          <t>kpi_pt Title 3</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -2302,29 +2302,29 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 2 Value</t>
+          <t>Label field: KPI 3 Title</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Tableau Bold 20pt</t>
+          <t>Tableau Semibold 8pt</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>#13233A</t>
+          <t>#5A6170</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Note 2</t>
+          <t>Value 3</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 2</t>
+          <t>kpi_pt Value 3</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -2334,29 +2334,29 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 2 Note</t>
+          <t>Label field: KPI 3 Value</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Tableau Book 8pt</t>
+          <t>Tableau Bold 20pt</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>#5A6170</t>
+          <t>#13233A</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Title 3</t>
+          <t>Note 3</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 3</t>
+          <t>kpi_pt Note 3</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 3 Title</t>
+          <t>Label field: KPI 3 Note</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Tableau Semibold 8pt</t>
+          <t>Tableau Book 8pt</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -2383,12 +2383,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Value 3</t>
+          <t>Title 4</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 3</t>
+          <t>kpi_pt Title 4</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -2398,29 +2398,29 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 3 Value</t>
+          <t>Label field: KPI 4 Title</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Tableau Bold 20pt</t>
+          <t>Tableau Semibold 8pt</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>#13233A</t>
+          <t>#5A6170</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Note 3</t>
+          <t>Value 4</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 3</t>
+          <t>kpi_pt Value 4</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -2430,29 +2430,29 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 3 Note</t>
+          <t>Label field: KPI 4 Value</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Tableau Book 8pt</t>
+          <t>Tableau Bold 20pt</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>#5A6170</t>
+          <t>#13233A</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Title 4</t>
+          <t>Note 4</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 4</t>
+          <t>kpi_pt Note 4</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -2462,12 +2462,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 4 Title</t>
+          <t>Label field: KPI 4 Note</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Tableau Semibold 8pt</t>
+          <t>Tableau Book 8pt</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2479,12 +2479,12 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Value 4</t>
+          <t>Title 5</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 4</t>
+          <t>kpi_pt Title 5</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -2494,29 +2494,29 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 4 Value</t>
+          <t>Label field: KPI 5 Title</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Tableau Bold 20pt</t>
+          <t>Tableau Semibold 8pt</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>#13233A</t>
+          <t>#5A6170</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Note 4</t>
+          <t>Value 5</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 4</t>
+          <t>kpi_pt Value 5</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -2526,29 +2526,29 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 4 Note</t>
+          <t>Label field: KPI 5 Value</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Tableau Book 8pt</t>
+          <t>Tableau Bold 20pt</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>#5A6170</t>
+          <t>#13233A</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Title 5</t>
+          <t>Note 5</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 5</t>
+          <t>kpi_pt Note 5</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -2558,12 +2558,12 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 5 Title</t>
+          <t>Label field: KPI 5 Note</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Tableau Semibold 8pt</t>
+          <t>Tableau Book 8pt</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2575,90 +2575,26 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Value 5</t>
+          <t>Check (top)</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 5</t>
+          <t>kpi_Check</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Circle, smallest, opacity 0%</t>
+          <t>Line, magenta, 2px</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 5 Value</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Tableau Bold 20pt</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>#13233A</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Note 5</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>kpi_pt Note 5</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Circle, smallest, opacity 0%</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Label field: KPI 5 Note</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Tableau Book 8pt</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>#5A6170</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Check (top)</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>kpi_Check</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Line, magenta, 2px</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
           <t>Calibration only; delete after</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
KPI cards: corner points fix the map extent, right alignment starts text at the anchor
</commit_message>
<xml_diff>
--- a/docs/Arcadia_KPI_Cards_Config.xlsx
+++ b/docs/Arcadia_KPI_Cards_Config.xlsx
@@ -1896,48 +1896,48 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>kpi_Frame</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>MAKELINE(MAKEPOINT([kpi_SheetH] / 2 * [kpi_Scale], -[kpi_SheetW] / 2 * [kpi_Scale]), MAKEPOINT(-[kpi_SheetH] / 2 * [kpi_Scale], [kpi_SheetW] / 2 * [kpi_Scale]))</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>0% opacity, no Fit</t>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>KPI 1 Title</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>"Closing headcount"</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>constant text for the title layer's Label shelf</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>kpi_Check</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>MAKELINE(MAKEPOINT(-([kpi_GridTop] + [kpi_CardH] - [kpi_SheetH] / 2) * [kpi_Scale] * [kpi_FitY], ([kpi_GridLeft] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]), MAKEPOINT(-([kpi_GridTop] - [kpi_SheetH] / 2) * [kpi_Scale] * [kpi_FitY], ([kpi_GridLeft] + 4 * ([kpi_CardW] + [kpi_GapX]) - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]))</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>calibration only</t>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>KPI 2 Title</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>"Closing FTE"</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>constant text for the title layer's Label shelf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>KPI 1 Title</t>
+          <t>KPI 3 Title</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>"Closing headcount"</t>
+          <t>"Hires"</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1949,12 +1949,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>KPI 2 Title</t>
+          <t>KPI 4 Title</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>"Closing FTE"</t>
+          <t>"Voluntary turnover (annualized)"</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1966,12 +1966,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>KPI 3 Title</t>
+          <t>KPI 5 Title</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>"Hires"</t>
+          <t>"Internal moves"</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1983,34 +1983,34 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>KPI 4 Title</t>
+          <t>kpi_Corner TL</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>"Voluntary turnover (annualized)"</t>
+          <t>MAKEPOINT([kpi_SheetH] / 2 * [kpi_Scale], -[kpi_SheetW] / 2 * [kpi_Scale])</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>constant text for the title layer's Label shelf</t>
+          <t>fixes the map extent; Circle, smallest, 0% opacity</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>KPI 5 Title</t>
+          <t>kpi_Corner BR</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>"Internal moves"</t>
+          <t>MAKEPOINT(-[kpi_SheetH] / 2 * [kpi_Scale], [kpi_SheetW] / 2 * [kpi_Scale])</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>constant text for the title layer's Label shelf</t>
+          <t>fixes the map extent; Circle, smallest, 0% opacity</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2071,36 +2071,44 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Frame</t>
+          <t>Title 1</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>kpi_Frame</t>
+          <t>kpi_pt Title 1</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>Circle, smallest, opacity 0%</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Opacity 0%, bottom layer</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr"/>
+          <t>Label field: KPI 1 Title</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Tableau Semibold 8pt</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>#5A6170</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Title 1</t>
+          <t>Value 1</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 1</t>
+          <t>kpi_pt Value 1</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -2110,29 +2118,29 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 1 Title</t>
+          <t>Label field: KPI 1 Value</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Tableau Semibold 8pt</t>
+          <t>Tableau Bold 20pt</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>#5A6170</t>
+          <t>#13233A</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Value 1</t>
+          <t>Note 1</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 1</t>
+          <t>kpi_pt Note 1</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -2142,29 +2150,29 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 1 Value</t>
+          <t>Label fields on one line: KPI 1 Note Up, KPI 1 Note Down, KPI 1 Note Flat</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Tableau Bold 20pt</t>
+          <t>Tableau Book 8pt</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>#13233A</t>
+          <t>Up #006B66 / Down #B8401F / Flat #5A6170 (color each field)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Note 1</t>
+          <t>Title 2</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 1</t>
+          <t>kpi_pt Title 2</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -2174,29 +2182,29 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Label fields on one line: KPI 1 Note Up, KPI 1 Note Down, KPI 1 Note Flat</t>
+          <t>Label field: KPI 2 Title</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Tableau Book 8pt</t>
+          <t>Tableau Semibold 8pt</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Up #006B66 / Down #B8401F / Flat #5A6170 (color each field)</t>
+          <t>#5A6170</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Title 2</t>
+          <t>Value 2</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 2</t>
+          <t>kpi_pt Value 2</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -2206,29 +2214,29 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 2 Title</t>
+          <t>Label field: KPI 2 Value</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Tableau Semibold 8pt</t>
+          <t>Tableau Bold 20pt</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>#5A6170</t>
+          <t>#13233A</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Value 2</t>
+          <t>Note 2</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 2</t>
+          <t>kpi_pt Note 2</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -2238,29 +2246,29 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 2 Value</t>
+          <t>Label field: KPI 2 Note</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Tableau Bold 20pt</t>
+          <t>Tableau Book 8pt</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>#13233A</t>
+          <t>#5A6170</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Note 2</t>
+          <t>Title 3</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 2</t>
+          <t>kpi_pt Title 3</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -2270,12 +2278,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 2 Note</t>
+          <t>Label field: KPI 3 Title</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Tableau Book 8pt</t>
+          <t>Tableau Semibold 8pt</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -2287,12 +2295,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Title 3</t>
+          <t>Value 3</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 3</t>
+          <t>kpi_pt Value 3</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -2302,29 +2310,29 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 3 Title</t>
+          <t>Label field: KPI 3 Value</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Tableau Semibold 8pt</t>
+          <t>Tableau Bold 20pt</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>#5A6170</t>
+          <t>#13233A</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Value 3</t>
+          <t>Note 3</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 3</t>
+          <t>kpi_pt Note 3</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -2334,29 +2342,29 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 3 Value</t>
+          <t>Label field: KPI 3 Note</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Tableau Bold 20pt</t>
+          <t>Tableau Book 8pt</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>#13233A</t>
+          <t>#5A6170</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Note 3</t>
+          <t>Title 4</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 3</t>
+          <t>kpi_pt Title 4</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -2366,12 +2374,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 3 Note</t>
+          <t>Label field: KPI 4 Title</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Tableau Book 8pt</t>
+          <t>Tableau Semibold 8pt</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -2383,12 +2391,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Title 4</t>
+          <t>Value 4</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 4</t>
+          <t>kpi_pt Value 4</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -2398,29 +2406,29 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 4 Title</t>
+          <t>Label field: KPI 4 Value</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Tableau Semibold 8pt</t>
+          <t>Tableau Bold 20pt</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>#5A6170</t>
+          <t>#13233A</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Value 4</t>
+          <t>Note 4</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 4</t>
+          <t>kpi_pt Note 4</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -2430,29 +2438,29 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 4 Value</t>
+          <t>Label field: KPI 4 Note</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Tableau Bold 20pt</t>
+          <t>Tableau Book 8pt</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>#13233A</t>
+          <t>#5A6170</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Note 4</t>
+          <t>Title 5</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 4</t>
+          <t>kpi_pt Title 5</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -2462,12 +2470,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 4 Note</t>
+          <t>Label field: KPI 5 Title</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Tableau Book 8pt</t>
+          <t>Tableau Semibold 8pt</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2479,12 +2487,12 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Title 5</t>
+          <t>Value 5</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 5</t>
+          <t>kpi_pt Value 5</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -2494,29 +2502,29 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 5 Title</t>
+          <t>Label field: KPI 5 Value</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Tableau Semibold 8pt</t>
+          <t>Tableau Bold 20pt</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>#5A6170</t>
+          <t>#13233A</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Value 5</t>
+          <t>Note 5</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 5</t>
+          <t>kpi_pt Note 5</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -2526,75 +2534,83 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Label field: KPI 5 Value</t>
+          <t>Label field: KPI 5 Note</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Tableau Bold 20pt</t>
+          <t>Tableau Book 8pt</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>#13233A</t>
+          <t>#5A6170</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Note 5</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>kpi_pt Note 5</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Corner TL</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>kpi_Corner TL</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>Circle, smallest, opacity 0%</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Label field: KPI 5 Note</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Tableau Book 8pt</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>#5A6170</t>
-        </is>
-      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>(no label)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Check (top)</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>kpi_Check</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Line, magenta, 2px</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Calibration only; delete after</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Corner BR</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>kpi_Corner BR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Circle, smallest, opacity 0%</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>(no label)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ALL text layers</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Alignment: Horizontal Right, Vertical Middle (Right makes the text start at the point)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
KPI cards: colored percentage on card 1 note, whole-number FTE, roomier row spacing
</commit_message>
<xml_diff>
--- a/docs/Arcadia_KPI_Cards_Config.xlsx
+++ b/docs/Arcadia_KPI_Cards_Config.xlsx
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>IF [K Valid] AND [K Net Pct] &gt; 0 THEN "+" + [K Net Pct Str] + " vs " + [K Open Str] + " at start" END</t>
+          <t>IF [K Valid] AND [K Net Pct] &gt; 0 THEN "+" + [K Net Pct Str] END</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>IF [K Valid] AND [K Net Pct] &lt; 0 THEN "−" + [K Net Pct Str] + " vs " + [K Open Str] + " at start" END</t>
+          <t>IF [K Valid] AND [K Net Pct] &lt; 0 THEN "−" + [K Net Pct Str] END</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>IF [K Valid] AND [K Net Pct] = 0 THEN [K Net Pct Str] + " vs " + [K Open Str] + " at start" END</t>
+          <t>IF [K Valid] AND [K Net Pct] = 0 THEN [K Net Pct Str] END</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1371,35 +1371,49 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>KPI 2 Value</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>IF NOT [K Valid] THEN "—" ELSE
-  IF DIV(INT(ROUND([K Close FTE] * 10, 0)), 10) &gt;= 1000
-  THEN STR(DIV(DIV(INT(ROUND([K Close FTE] * 10, 0)), 10), 1000)) + "," +
-       RIGHT("00" + STR(DIV(INT(ROUND([K Close FTE] * 10, 0)), 10) % 1000), 3)
-  ELSE STR(DIV(INT(ROUND([K Close FTE] * 10, 0)), 10)) END
-  + "." + STR(INT(ROUND([K Close FTE] * 10, 0)) % 10)
-END</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>12,940.0: round to tenths, then split whole and tenth</t>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>KPI 1 Note Rest</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IF [K Valid] THEN "vs " + [K Open Str] + " at start" END</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>slate, Tableau Book</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>KPI 2 Value</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>IF NOT [K Valid] THEN "—"
+ELSEIF ROUND([K Close FTE], 0) &gt;= 1000
+THEN STR(DIV(INT(ROUND([K Close FTE], 0)), 1000)) + "," + RIGHT("00" + STR(INT(ROUND([K Close FTE], 0)) % 1000), 3)
+ELSE STR(INT(ROUND([K Close FTE], 0))) END</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>12,940.0: round to tenths, then split whole and tenth</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>KPI 2 Note</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>IF NOT [K Valid] THEN "" ELSE
   IF INT(ROUND([K Part Time Gap], 0)) &gt;= 1000
@@ -1410,15 +1424,15 @@
 END</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>KPI 3 Value</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>IF NOT [K Valid] THEN "—"
 ELSEIF [K Hires] &gt;= 1000
@@ -1426,19 +1440,19 @@
 ELSE STR(INT([K Hires])) END</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>the comma pattern on [K Hires]</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>KPI 3 Note</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>IF NOT [K Valid] THEN "" ELSE
   STR(DIV(INT(ROUND(ZN([Hire Rate (annualized)]) * 1000, 0)), 10)) + "." +
@@ -1446,19 +1460,19 @@
 END</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>the percent pattern on the annualized hire rate</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>KPI 4 Value</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>IF NOT [K Valid] OR [Average Headcount] &lt; 20 THEN "—" ELSE
   STR(DIV(INT(ROUND([Voluntary Turnover (annualized)] * 1000, 0)), 10)) + "." +
@@ -1466,19 +1480,19 @@
 END</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>hidden for groups under 20 people, like Rate Shown</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>KPI 4 Note</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>IF NOT [K Valid] THEN "" ELSE
   IF [K Leavers Vol] &gt;= 1000
@@ -1488,19 +1502,19 @@
 END</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>the comma pattern on [K Leavers Vol]</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>KPI 5 Value</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>IF NOT [K Valid] THEN "—"
 ELSEIF [K Moves] &gt;= 1000
@@ -1508,19 +1522,19 @@
 ELSE STR(INT([K Moves])) END</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>the comma pattern on [K Moves]</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>KPI 5 Note</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>IF NOT [K Valid] THEN "" ELSE
   IF [K Promotions] &gt;= 1000
@@ -1534,30 +1548,17 @@
 END</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>kpi_lat Title</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>-([kpi_GridTop] + [kpi_TitleDY] + [kpi_ShiftY] - [kpi_SheetH] / 2) * [kpi_Scale] * [kpi_FitY]</t>
-        </is>
-      </c>
       <c r="C27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>kpi_lat Value</t>
+          <t>kpi_lat Title</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>-([kpi_GridTop] + [kpi_ValueDY] + [kpi_ShiftY] - [kpi_SheetH] / 2) * [kpi_Scale] * [kpi_FitY]</t>
+          <t>-([kpi_GridTop] + [kpi_TitleDY] + [kpi_ShiftY] - [kpi_SheetH] / 2) * [kpi_Scale] * [kpi_FitY]</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr"/>
@@ -1565,12 +1566,12 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>kpi_lat Sub</t>
+          <t>kpi_lat Value</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>-([kpi_GridTop] + [kpi_SubDY] + [kpi_ShiftY] - [kpi_SheetH] / 2) * [kpi_Scale] * [kpi_FitY]</t>
+          <t>-([kpi_GridTop] + [kpi_ValueDY] + [kpi_ShiftY] - [kpi_SheetH] / 2) * [kpi_Scale] * [kpi_FitY]</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr"/>
@@ -1578,12 +1579,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>kpi_lon C1</t>
+          <t>kpi_lat Sub</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>([kpi_GridLeft] + 0 * ([kpi_CardW] + [kpi_GapX]) + [kpi_PadX] + [kpi_ShiftX] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]</t>
+          <t>-([kpi_GridTop] + [kpi_SubDY] + [kpi_ShiftY] - [kpi_SheetH] / 2) * [kpi_Scale] * [kpi_FitY]</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr"/>
@@ -1591,12 +1592,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>kpi_lon C2</t>
+          <t>kpi_lon C1</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>([kpi_GridLeft] + 1 * ([kpi_CardW] + [kpi_GapX]) + [kpi_PadX] + [kpi_ShiftX] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]</t>
+          <t>([kpi_GridLeft] + 0 * ([kpi_CardW] + [kpi_GapX]) + [kpi_PadX] + [kpi_ShiftX] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr"/>
@@ -1604,12 +1605,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>kpi_lon C3</t>
+          <t>kpi_lon C2</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>([kpi_GridLeft] + 2 * ([kpi_CardW] + [kpi_GapX]) + [kpi_PadX] + [kpi_ShiftX] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]</t>
+          <t>([kpi_GridLeft] + 1 * ([kpi_CardW] + [kpi_GapX]) + [kpi_PadX] + [kpi_ShiftX] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr"/>
@@ -1617,12 +1618,12 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>kpi_lon C4</t>
+          <t>kpi_lon C3</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>([kpi_GridLeft] + 3 * ([kpi_CardW] + [kpi_GapX]) + [kpi_PadX] + [kpi_ShiftX] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]</t>
+          <t>([kpi_GridLeft] + 2 * ([kpi_CardW] + [kpi_GapX]) + [kpi_PadX] + [kpi_ShiftX] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr"/>
@@ -1630,12 +1631,12 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>kpi_lon C5</t>
+          <t>kpi_lon C4</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>([kpi_GridLeft] + 4 * ([kpi_CardW] + [kpi_GapX]) + [kpi_PadX] + [kpi_ShiftX] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]</t>
+          <t>([kpi_GridLeft] + 3 * ([kpi_CardW] + [kpi_GapX]) + [kpi_PadX] + [kpi_ShiftX] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr"/>
@@ -1643,29 +1644,25 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 1</t>
+          <t>kpi_lon C5</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Title], [kpi_lon C1])</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>anchor point (Note uses kpi_lat Sub)</t>
-        </is>
-      </c>
+          <t>([kpi_GridLeft] + 4 * ([kpi_CardW] + [kpi_GapX]) + [kpi_PadX] + [kpi_ShiftX] - [kpi_SheetW] / 2) * [kpi_Scale] * [kpi_FitX]</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 2</t>
+          <t>kpi_pt Title 1</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Title], [kpi_lon C2])</t>
+          <t>MAKEPOINT([kpi_lat Title], [kpi_lon C1])</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -1677,12 +1674,12 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 3</t>
+          <t>kpi_pt Title 2</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Title], [kpi_lon C3])</t>
+          <t>MAKEPOINT([kpi_lat Title], [kpi_lon C2])</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -1694,12 +1691,12 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 4</t>
+          <t>kpi_pt Title 3</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Title], [kpi_lon C4])</t>
+          <t>MAKEPOINT([kpi_lat Title], [kpi_lon C3])</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -1711,12 +1708,12 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Title 5</t>
+          <t>kpi_pt Title 4</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Title], [kpi_lon C5])</t>
+          <t>MAKEPOINT([kpi_lat Title], [kpi_lon C4])</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -1728,12 +1725,12 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 1</t>
+          <t>kpi_pt Title 5</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Value], [kpi_lon C1])</t>
+          <t>MAKEPOINT([kpi_lat Title], [kpi_lon C5])</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -1745,12 +1742,12 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 2</t>
+          <t>kpi_pt Value 1</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Value], [kpi_lon C2])</t>
+          <t>MAKEPOINT([kpi_lat Value], [kpi_lon C1])</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -1762,12 +1759,12 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 3</t>
+          <t>kpi_pt Value 2</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Value], [kpi_lon C3])</t>
+          <t>MAKEPOINT([kpi_lat Value], [kpi_lon C2])</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1779,12 +1776,12 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 4</t>
+          <t>kpi_pt Value 3</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Value], [kpi_lon C4])</t>
+          <t>MAKEPOINT([kpi_lat Value], [kpi_lon C3])</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -1796,12 +1793,12 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Value 5</t>
+          <t>kpi_pt Value 4</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Value], [kpi_lon C5])</t>
+          <t>MAKEPOINT([kpi_lat Value], [kpi_lon C4])</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -1813,12 +1810,12 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 1</t>
+          <t>kpi_pt Value 5</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Sub], [kpi_lon C1])</t>
+          <t>MAKEPOINT([kpi_lat Value], [kpi_lon C5])</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -1830,12 +1827,12 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 2</t>
+          <t>kpi_pt Note 1</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Sub], [kpi_lon C2])</t>
+          <t>MAKEPOINT([kpi_lat Sub], [kpi_lon C1])</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -1847,12 +1844,12 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 3</t>
+          <t>kpi_pt Note 2</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Sub], [kpi_lon C3])</t>
+          <t>MAKEPOINT([kpi_lat Sub], [kpi_lon C2])</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1864,12 +1861,12 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>kpi_pt Note 4</t>
+          <t>kpi_pt Note 3</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_lat Sub], [kpi_lon C4])</t>
+          <t>MAKEPOINT([kpi_lat Sub], [kpi_lon C3])</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -1881,46 +1878,46 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
+          <t>kpi_pt Note 4</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>MAKEPOINT([kpi_lat Sub], [kpi_lon C4])</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>anchor point (Note uses kpi_lat Sub)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
           <t>kpi_pt Note 5</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>MAKEPOINT([kpi_lat Sub], [kpi_lon C5])</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>anchor point (Note uses kpi_lat Sub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>KPI 1 Title</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>"Closing headcount"</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>constant text for the title layer's Label shelf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>KPI 2 Title</t>
+          <t>KPI 1 Title</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>"Closing FTE"</t>
+          <t>"Closing headcount"</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1932,12 +1929,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>KPI 3 Title</t>
+          <t>KPI 2 Title</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>"Hires"</t>
+          <t>"Closing FTE"</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1949,12 +1946,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>KPI 4 Title</t>
+          <t>KPI 3 Title</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>"Voluntary turnover (annualized)"</t>
+          <t>"Hires"</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1966,12 +1963,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>KPI 5 Title</t>
+          <t>KPI 4 Title</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>"Internal moves"</t>
+          <t>"Voluntary turnover (annualized)"</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1983,32 +1980,49 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>kpi_Corner TL</t>
+          <t>KPI 5 Title</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MAKEPOINT([kpi_SheetH] / 2 * [kpi_Scale], -[kpi_SheetW] / 2 * [kpi_Scale])</t>
+          <t>"Internal moves"</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>fixes the map extent; Circle, smallest, 0% opacity</t>
+          <t>constant text for the title layer's Label shelf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>kpi_Corner TL</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>MAKEPOINT([kpi_SheetH] / 2 * [kpi_Scale], -[kpi_SheetW] / 2 * [kpi_Scale])</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>fixes the map extent; Circle, smallest, 0% opacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>kpi_Corner BR</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>MAKEPOINT(-[kpi_SheetH] / 2 * [kpi_Scale], [kpi_SheetW] / 2 * [kpi_Scale])</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>fixes the map extent; Circle, smallest, 0% opacity</t>
         </is>
@@ -2150,7 +2164,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Label fields on one line: KPI 1 Note Up, KPI 1 Note Down, KPI 1 Note Flat</t>
+          <t>Label line: &lt;KPI 1 Note Up&gt;&lt;KPI 1 Note Down&gt;&lt;KPI 1 Note Flat&gt; &lt;KPI 1 Note Rest&gt; (typed space before Rest)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -2160,7 +2174,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Up #006B66 / Down #B8401F / Flat #5A6170 (color each field)</t>
+          <t>Up #006B66 / Down #B8401F / Flat #5A6170 / Rest #5A6170 (color each field)</t>
         </is>
       </c>
     </row>
@@ -2569,8 +2583,6 @@
           <t>(no label)</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2593,8 +2605,6 @@
           <t>(no label)</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2602,15 +2612,11 @@
           <t>ALL text layers</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>Alignment: Horizontal Right, Vertical Middle (Right makes the text start at the point)</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2775,7 +2781,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>12,940.0</t>
+          <t>12,940</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -2835,6 +2841,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
KPI cards guide: full dashboard grid with header, KPI band and chart slots
</commit_message>
<xml_diff>
--- a/docs/Arcadia_KPI_Cards_Config.xlsx
+++ b/docs/Arcadia_KPI_Cards_Config.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Layers" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grid" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2841,11 +2842,468 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
           <t>Range: Start Month 2025-07-31, End Month 2026-06-30. Start after End: every value shows an em dash.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Header band</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Blank</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1400</v>
+      </c>
+      <c r="G2" t="n">
+        <v>76</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Background #13233A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Logo</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>56</v>
+      </c>
+      <c r="E3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F3" t="n">
+        <v>177</v>
+      </c>
+      <c r="G3" t="n">
+        <v>48</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>arcadia_logo_horizontal_reverse.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Title and subtitle</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>256</v>
+      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="n">
+        <v>470</v>
+      </c>
+      <c r="G4" t="n">
+        <v>58</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>White title; subtitle #C9D1DC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Start Month</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Parameter control</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>744</v>
+      </c>
+      <c r="E5" t="n">
+        <v>22</v>
+      </c>
+      <c r="F5" t="n">
+        <v>140</v>
+      </c>
+      <c r="G5" t="n">
+        <v>32</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Compact dropdown, white bg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>End Month</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Parameter control</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>892</v>
+      </c>
+      <c r="E6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F6" t="n">
+        <v>140</v>
+      </c>
+      <c r="G6" t="n">
+        <v>32</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Headcount / FTE pills</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sheet (Measure Toggle)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1044</v>
+      </c>
+      <c r="E7" t="n">
+        <v>22</v>
+      </c>
+      <c r="F7" t="n">
+        <v>150</v>
+      </c>
+      <c r="G7" t="n">
+        <v>32</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Methodology pill</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1204</v>
+      </c>
+      <c r="E8" t="n">
+        <v>22</v>
+      </c>
+      <c r="F8" t="n">
+        <v>140</v>
+      </c>
+      <c r="G8" t="n">
+        <v>32</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KPI card background</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>78</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1400</v>
+      </c>
+      <c r="G9" t="n">
+        <v>110</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>arcadia_kpi_cards_bg.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KPI cards</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>78</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1400</v>
+      </c>
+      <c r="G10" t="n">
+        <v>110</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>above the image</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Waterfall card</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sheet or Blank</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>56</v>
+      </c>
+      <c r="E11" t="n">
+        <v>188</v>
+      </c>
+      <c r="F11" t="n">
+        <v>780</v>
+      </c>
+      <c r="G11" t="n">
+        <v>624</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Headcount trend card</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sheet or Blank</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>848</v>
+      </c>
+      <c r="E12" t="n">
+        <v>188</v>
+      </c>
+      <c r="F12" t="n">
+        <v>496</v>
+      </c>
+      <c r="G12" t="n">
+        <v>300</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Turnover by function card</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sheet or Blank</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>848</v>
+      </c>
+      <c r="E13" t="n">
+        <v>500</v>
+      </c>
+      <c r="F13" t="n">
+        <v>496</v>
+      </c>
+      <c r="G13" t="n">
+        <v>312</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Footer note</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>56</v>
+      </c>
+      <c r="E14" t="n">
+        <v>820</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1288</v>
+      </c>
+      <c r="G14" t="n">
+        <v>22</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Slate #5A6170, 8 pt</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Headcount walk guide: dynamic waterfall title and caption (FIXED calcs); caption slot in the dashboard grid
</commit_message>
<xml_diff>
--- a/docs/Arcadia_KPI_Cards_Config.xlsx
+++ b/docs/Arcadia_KPI_Cards_Config.xlsx
@@ -2860,7 +2860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3069,7 +3069,6 @@
       <c r="G6" t="n">
         <v>32</v>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -3097,7 +3096,6 @@
       <c r="G7" t="n">
         <v>32</v>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -3125,7 +3123,6 @@
       <c r="G8" t="n">
         <v>32</v>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -3217,7 +3214,6 @@
       <c r="G11" t="n">
         <v>624</v>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -3245,7 +3241,6 @@
       <c r="G12" t="n">
         <v>300</v>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -3273,11 +3268,10 @@
       <c r="G13" t="n">
         <v>312</v>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -3304,6 +3298,38 @@
       <c r="H14" t="inlineStr">
         <is>
           <t>Slate #5A6170, 8 pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Waterfall caption</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>68</v>
+      </c>
+      <c r="E15" t="n">
+        <v>756</v>
+      </c>
+      <c r="F15" t="n">
+        <v>756</v>
+      </c>
+      <c r="G15" t="n">
+        <v>48</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Over the waterfall card's bottom padding; waterfall sheet bottom inner padding 64</t>
         </is>
       </c>
     </row>

</xml_diff>